<commit_message>
Add first 23 verified records to the database (v0.3.0)
Covers all 8 categories with stable fields (name, organizer, official
URL, format, country/region) verified against each program's official
website. Deadline/event-date fields left as UNKNOWN since they change
annually; see Notes per record.
</commit_message>
<xml_diff>
--- a/database/AcademicAtlas.xlsx
+++ b/database/AcademicAtlas.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -528,6 +528,1777 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>COMP-0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>International competitions</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>International Mathematical Olympiad (IMO)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>International Mathematical Olympiad Foundation</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>National team selection required; pre-university students</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Annual international mathematics competition for pre-university students, held since 1959; national teams compete in two exam papers.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://www.imo-official.org/</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Free (national selection process varies by country)</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Team selection is handled by each country's national olympiad committee, not centrally; host country/dates change yearly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>COMP-0002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>International competitions</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>International Physics Olympiad (IPhO)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>International Physics Olympiad Organization</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>National team selection required; pre-university students</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Annual international physics competition for secondary school students, held since 1967.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>https://www.ipho-new.org/</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Free (national selection process varies by country)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Selection handled nationally; host country/dates change yearly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>COMP-0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>International competitions</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>International Chemistry Olympiad (IChO)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>International Chemistry Olympiad International Information Centre</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>National team selection required; secondary school students</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Annual international chemistry competition held since 1968, combining theoretical and experimental exams.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://www.icho-official.org/</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Free (national selection process varies by country)</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Selection handled nationally; host country/dates change yearly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>COMP-0004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>International competitions</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>International Olympiad in Informatics (IOI)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>IOI General Assembly</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>National team selection required; pre-university students</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Annual international programming/algorithms competition for secondary school students, held since 1989.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://ioinformatics.org/</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Free (national selection process varies by country)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Selection handled nationally; host country/dates change yearly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>COMP-0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>International competitions</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>International Biology Olympiad (IBO)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>International Biology Olympiad e.V.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>National team selection required; pre-university students under 20</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Annual international biology competition for secondary school students, held since 1990.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://www.ibo-info.org/en/</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Free (national selection process varies by country)</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Selection handled nationally; host country/dates change yearly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>COMP-0006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>International competitions</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Regeneron International Science and Engineering Fair (ISEF)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Society for Science</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Must first win at a Society-affiliated local/regional/state/national science fair</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>World's largest international pre-college science competition; finalists qualify through affiliated fairs in 60+ countries, regions, and territories.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://www.societyforscience.org/isef/</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Free to compete (affiliate fair/travel costs vary)</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Entry is via affiliated local fairs, not direct application; affiliate fair deadlines vary by region.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>COMP-0007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>International competitions</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>John Locke Institute Essay Competition (Global Essay Prize)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>John Locke Institute</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Open globally; no age restriction stated</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Annual essay competition across philosophy, politics, economics, history, psychology, theology, and law; participants from 100+ countries.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://www.johnlockeinstitute.com/</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Deadline changes annually; check official site for current cycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>COMP-0008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>International competitions</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>World Scholar's Cup</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>World Scholar's Cup</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Teams of three students; three age divisions</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Global academic competition combining a quiz bowl, collaborative writing, team debate, and a Tournament of Champions at Yale University; regional rounds in 70+ countries.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://www.scholarscup.org/</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Regional round dates/fees vary by location; check local round listing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>RES-0001</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Research programs / opportunities</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Research Science Institute (RSI)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Center for Excellence in Education (CEE), hosted at MIT</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>United States (international students apply via home-country selection)</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>US students with one year left before high school graduation (seniors not eligible); international applicants apply through their own country's selection process</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Free 6-week on-campus summer research program combining STEM coursework with mentored research; approximately 100 students selected annually.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://www.cee.org/programs/research-science-institute</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>International admission runs through separate national selection procedures with their own timelines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RES-0002</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Research programs / opportunities</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>PRIMES (Program for Research in Mathematics, Engineering and Science for High School Students)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>MIT Department of Mathematics</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>High school sophomores/juniors; specific grades vary by track (MIT PRIMES, PRIMES-USA, PRIMES Circle, Yulia's Dream)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Year-long mentored research program in mathematics, computer science, and computational biology for high school students.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://math.mit.edu/research/highschool/primes/</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Multiple tracks with different eligibility/geography; see official site for the specific track.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RES-0003</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Research programs / opportunities</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Simons Summer Research Program</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Stony Brook University</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>US citizens/permanent residents; high school juniors, at least 16 by program start, nominated by their school</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>7-week mentored research program pairing approximately 40 selected high school students with Stony Brook University faculty.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://www.stonybrook.edu/simons/</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Requires school nomination (max 2 per school); highly selective (~5% acceptance rate).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>SUM-0001</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Summer schools</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Summer Science Program (SSP)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SSP International (nonprofit)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>High school juniors</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>5-week residential summer research program in astrophysics, biochemistry, bacterial genomics, or synthetic chemistry, held on partner college campuses.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://ssp.org/</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>UNKNOWN (see Fees &amp; Financial Aid page)</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Cost varies by track/campus; need-based financial aid available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SUM-0002</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Summer schools</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Yale Young Global Scholars (YYGS)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Yale University</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>High school students from around the world (150+ countries)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Two-week residential summer sessions at Yale across three tracks: Innovations in Science &amp; Technology, Politics of Law &amp; Economics, and Solving Global Challenges.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://globalscholars.yale.edu/</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Paid (need-based financial aid and scholarships available)</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Tuition varies by session; see site for current pricing and aid options.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SUM-0003</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Summer schools</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MITES (MIT Introduction to Technology, Engineering, and Science)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Massachusetts Institute of Technology</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>United States (MITES Saturdays limited to Boston/Cambridge/Lawrence, MA)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>US citizens/permanent residents, 11th grade, for MITES Summer/Semester; MITES Saturdays limited to Boston-area public school students grades 7-10</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Free residential (Summer) or remote (Semester) STEM enrichment program at MIT for underrepresented high school students.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://mites.mit.edu/</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Free (students only cover transportation)</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Multiple program tracks (Summer/Semester/Saturdays) with different eligibility and formats.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SCHOL-0001</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Scholarships</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Davis United World College Scholars Program</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Administered by Middlebury College (founded by Shelby Davis and Phil Geier)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>International (for UWC graduates attending US universities)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Graduates of the 18 United World College (UWC) high schools</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Need-based financial aid for UWC graduates pursuing higher education at 100+ partner colleges/universities in the United States.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>https://www.davisuwcscholars.org/</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Need-based (amount varies)</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Only open to UWC graduates, not the general public.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SCHOL-0002</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Scholarships</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>QuestBridge National College Match</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>QuestBridge</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>High-achieving high school seniors from low-income backgrounds</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Matches selected students with full four-year scholarships at QuestBridge partner colleges.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>https://www.questbridge.org/</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Full four-year scholarship (need-based)</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Applicants rank partner colleges; matches are binding at some partners, similar to Early Decision.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>COURSE-0001</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Academic courses</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Center for Talented Youth (CTY)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Johns Hopkins University</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>United States (online option available internationally)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Grades 2-12; qualification via standardized test scores (e.g., 95th+ percentile for Advanced CTY Level)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Academic enrichment courses (in-person and online) for advanced learners, spanning STEM and humanities subjects.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>https://cty.jhu.edu/</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Paid, varies by course (e.g., ~$7,801 for a residential course); need-based financial aid available; $15 application fee</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Tuition varies significantly by course/length; see course catalog for exact pricing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>COURSE-0002</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Academic courses</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Stanford Online High School</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Stanford University (Stanford Pre-Collegiate Studies)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>International (fully online)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Academically advanced students, grades 7-12</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Accredited, fully online private high school with live seminar-style classes; awards approximately $2.5M annually in financial aid.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>https://onlinehighschool.stanford.edu/</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Paid (financial aid available)</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Full diploma-granting school, not a single course; admissions is selective.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>INNOV-0001</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Innovation challenges</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Conrad Challenge</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Conrad Foundation</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Ages 13-18, teams of 2-5 students</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Multi-stage innovation/entrepreneurship competition where student teams design solutions to real-world problems, culminating in an in-person Innovation Summit.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>https://www.conradchallenge.org/</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Free to start (Activation/Lean Canvas stages); $499/team for Innovation Stage; $499/person for in-person Summit; financial aid available</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Costs apply only at later stages; discounts available for Title I schools.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>INNOV-0002</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Innovation challenges</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Technovation Girls</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Technovation (nonprofit)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Girls/underrepresented genders in tech, team-based</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Global technology entrepreneurship program where student teams build mobile/AI solutions to community problems.</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>https://www.technovation.org/</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Program registration is managed via technovationchallenge.org; confirm current eligibility there.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>JOUR-0001</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Academic journals &amp; publications</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>The Concord Review</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>The Concord Review, Inc.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Secondary school students (history research papers)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Quarterly journal publishing academic history research papers written by secondary school students; also operates the National Writing Board assessment service.</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>https://www.tcr.org/</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Typical submission is a long-form (~5,000+ word) history research paper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>JOUR-0002</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Academic journals &amp; publications</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Journal of Student Research (High School Edition)</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Journal of Student Research (Houston, TX)</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>First author must be a high school student (grades 9-12) with a listed teacher/advisor</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Peer-reviewed, open-access multidisciplinary journal publishing high school, undergraduate, and graduate student research (AP Research, IB, honors research, etc.).</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>https://www.jsr.org/</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Paid Article Processing Charge: $50 at submission + $299 after acceptance</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Double-blind peer review; APC charged in two phases.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CONF-0001</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Conferences &amp; academic events</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Harvard Model United Nations (HMUN)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Harvard College (student-run)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>International</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>High school students; delegations from 60+ countries</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Large in-person Model UN conference held in Boston, run by Harvard undergraduates, simulating international diplomacy committees.</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://www.harvardmun.org/</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>In-person</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Held annually in late January; check official site for current session dates/fees.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Subject taxonomy + Typical_Window fields; tag all 53 records
Schema (v0.8.0 groundwork, Discoverability + Freshness):
* New column 18 `Subject` (required, multi-value, ';'-separated) drawn
  from a 15-value controlled vocabulary documented in
  docs/DatabaseSchema.md and enforced by scripts/validate.py (unknown
  value / duplicate / stray-';' checks).
* New column 19 `Typical_Window` (optional) for the recurring
  month/season a program usually opens; left empty for now — it is
  filled during the official-source verification sweep, not guessed.
* Backfilled `Subject` for all 53 existing records; national qualifying
  stages carry the same subject(s) as the international final they feed.
* Regenerated docs/data.json (53 records); validate.py passes with 0
  errors. Added .gitignore (Python __pycache__, etc.).

No existing record was removed, renumbered, or otherwise altered.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/database/AcademicAtlas.xlsx
+++ b/database/AcademicAtlas.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q54"/>
+  <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -537,6 +537,16 @@
           <t>Qualifies_For</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Subject</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Typical_Window</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -619,6 +629,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -701,6 +716,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -783,6 +803,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -865,6 +890,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -947,6 +977,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1029,6 +1064,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1111,6 +1151,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>Writing; Social Sciences &amp; Humanities; Economics &amp; Business</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1193,6 +1238,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1275,6 +1325,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1357,6 +1412,11 @@
           <t>US only</t>
         </is>
       </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>Mathematics; Computer Science</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1439,6 +1499,11 @@
           <t>US only</t>
         </is>
       </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1521,6 +1586,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Earth &amp; Space; Biology; Chemistry</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1603,6 +1673,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1685,6 +1760,11 @@
           <t>US only</t>
         </is>
       </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Engineering &amp; Robotics; Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1767,6 +1847,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1849,6 +1934,11 @@
           <t>US only</t>
         </is>
       </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1931,6 +2021,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2013,6 +2108,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2095,6 +2195,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>Engineering &amp; Robotics; Economics &amp; Business</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2177,6 +2282,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>Computer Science; Economics &amp; Business</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2259,6 +2369,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Social Sciences &amp; Humanities; Writing</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2341,6 +2456,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2423,6 +2543,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>Social Sciences &amp; Humanities</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2505,6 +2630,11 @@
           <t>US only</t>
         </is>
       </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2587,6 +2717,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2669,6 +2804,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>Economics &amp; Business</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2751,6 +2891,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>Environment; Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2833,6 +2978,11 @@
           <t>US only</t>
         </is>
       </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2915,6 +3065,11 @@
           <t>US only</t>
         </is>
       </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2997,6 +3152,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3079,6 +3239,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3161,6 +3326,11 @@
           <t>US only</t>
         </is>
       </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3243,6 +3413,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3325,6 +3500,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3407,6 +3587,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3489,6 +3674,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3571,6 +3761,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>Earth &amp; Space; Physics</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3653,6 +3848,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>Linguistics</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3735,6 +3935,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Earth &amp; Space; Social Sciences &amp; Humanities</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3817,6 +4022,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3899,6 +4109,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3981,6 +4196,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>Engineering &amp; Robotics</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4063,6 +4283,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>Social Sciences &amp; Humanities</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4145,6 +4370,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>Social Sciences &amp; Humanities</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4227,6 +4457,11 @@
           <t>International</t>
         </is>
       </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4314,6 +4549,11 @@
           <t>COMP-0001</t>
         </is>
       </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4401,6 +4641,11 @@
           <t>COMP-0002</t>
         </is>
       </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4488,6 +4733,11 @@
           <t>COMP-0003</t>
         </is>
       </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4575,6 +4825,11 @@
           <t>COMP-0004</t>
         </is>
       </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4662,6 +4917,11 @@
           <t>COMP-0005</t>
         </is>
       </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4749,6 +5009,11 @@
           <t>COMP-0011</t>
         </is>
       </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>Earth &amp; Space; Physics</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4836,6 +5101,11 @@
           <t>COMP-0013</t>
         </is>
       </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>Earth &amp; Space; Social Sciences &amp; Humanities</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4921,6 +5191,11 @@
       <c r="Q54" t="inlineStr">
         <is>
           <t>COMP-0006</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
         </is>
       </c>
     </row>
@@ -4935,7 +5210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5050,7 +5325,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
@@ -5108,6 +5382,198 @@
       <c r="B16" t="inlineStr">
         <is>
           <t>Optional column: ID of the international opportunity a national/regional stage feeds into.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Subjects</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Covers (Subject column; ';'-separated for multiple)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Mathematics</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Pure and applied mathematics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Physics</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Physics and astrophysics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Chemistry</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Chemistry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Biology</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Biology and the life sciences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Programming, informatics, algorithms, AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Engineering &amp; Robotics</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Engineering, robotics, hardware design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Earth &amp; Space</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Astronomy, geography, geology, earth sciences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Environmental science and sustainability.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Economics &amp; Business</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Economics, finance, entrepreneurship.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Social Sciences &amp; Humanities</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>History, philosophy, psychology, social sciences.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Linguistics</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Language and linguistics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Writing</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Essay, journalism, creative and academic writing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Arts &amp; Design</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Visual, performing, and design disciplines.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Medicine &amp; Health</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Medicine, public health, biomedical topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Interdisciplinary</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Spans multiple fields, or a general program.</t>
         </is>
       </c>
     </row>

</xml_diff>